<commit_message>
delete PMOC: not effective
</commit_message>
<xml_diff>
--- a/ui/src/assets/excel/template.xlsx
+++ b/ui/src/assets/excel/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Marriage-License-System\ui\src\assets\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D7FCD4-0EB0-49AD-B6EA-F8ABC384B3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8F226AE-588C-413B-A4F1-39B51A2B0BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" tabRatio="1000" firstSheet="4" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="APPLICATION" sheetId="1" r:id="rId1"/>
@@ -25,17 +25,7 @@
     <sheet name="Notice" sheetId="6" r:id="rId10"/>
     <sheet name="AddressBACKnotice" sheetId="16" r:id="rId11"/>
     <sheet name="EnvelopeAddress" sheetId="15" r:id="rId12"/>
-    <sheet name="PMOC" sheetId="17" r:id="rId13"/>
   </sheets>
-  <definedNames>
-    <definedName name="brideName" localSheetId="12">"brideName"</definedName>
-    <definedName name="cN" localSheetId="12">"cN"</definedName>
-    <definedName name="controlNumber" localSheetId="12">"controlNumber"</definedName>
-    <definedName name="date" localSheetId="12">"date"</definedName>
-    <definedName name="groomName" localSheetId="12">"groomName"</definedName>
-    <definedName name="yearToday" localSheetId="12">"yearToday"</definedName>
-    <definedName name="yerdeyt" localSheetId="12">"yerdeyt"</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1565,2223 +1555,6 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>75007</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>159640</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>34635</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="23" name="Picture 22">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{445D9F85-186B-4DF0-AAAA-84C3200C64FC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="75007" y="0"/>
-          <a:ext cx="7371258" cy="10321635"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>33618</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>131243</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>79663</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>138407</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="TextBox 23">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32DDF4FA-16FD-460E-B867-50D93C2B519F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="33618" y="442970"/>
-          <a:ext cx="7319681" cy="786482"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1000">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Republic of the Philippines</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1000">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Province of Nueva Vizcaya</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400" b="1">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>MUNICIPALITY OF SOLANO </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1000" b="1">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>	</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1000">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-            <a:ea typeface="+mn-ea"/>
-            <a:cs typeface="+mn-cs"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1000">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>National Highway, Barangay Roxas, Solano, Nueva Vizcaya, 3709</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:endParaRPr lang="en-US" sz="1000">
-            <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>63285</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>62478</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>167343</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>80409</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="25" name="Picture 24">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4663009A-28FB-4A08-A99B-B192142963A2}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5518512" y="218342"/>
-          <a:ext cx="1316331" cy="1264840"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>132407</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>46159</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>437357</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>110647</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="26" name="Picture 25">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C7816BAA-E8E0-4F84-9A3B-8DA335A19A78}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="738543" y="513750"/>
-          <a:ext cx="911087" cy="843806"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>33618</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>105782</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>75182</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>89329</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="27" name="TextBox 26">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E524575-09B4-4657-935F-416204A3ACD5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="33618" y="1820282"/>
-          <a:ext cx="7315200" cy="295274"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Rockwell Condensed" panose="02060603050405020104" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>CERTIFICATE OF COMPLIANCE</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>33619</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>88917</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>70248</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>40573</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="TextBox 27">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13A8CC8B-867A-4141-8974-0F0297973AF6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="33619" y="2115144"/>
-          <a:ext cx="7310265" cy="263384"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1400">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Rockwell Condensed" panose="02060603050405020104" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>PRE-MARRIAGE ORIENTATION AND COUNSELING (PMOC)</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1400">
-            <a:latin typeface="Rockwell Condensed" panose="02060603050405020104" pitchFamily="18" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>33619</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>35566</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>82510</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>78347</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="TextBox 28">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{21FFAD61-C550-4163-8026-E31DAF3BCC40}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="33619" y="2841111"/>
-          <a:ext cx="7322527" cy="198645"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" algn="ctr" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>This certifies that:</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>435967</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>80173</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>78861</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>56917</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="30" name="TextBox 29">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1986C17-4560-4F25-A7BE-7B90BD33D4F5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1042103" y="3353309"/>
-          <a:ext cx="855167" cy="288472"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="1">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>GROOM</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>: </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>45334</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>96913</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>176745</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>68678</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="31" name="TextBox 30">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4666BFB3-33A1-44AE-BBE3-15723622BB87}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4288289" y="3370049"/>
-          <a:ext cx="737547" cy="283493"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="1">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>BRIDE</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>:</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>561875</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>85775</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>7530</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>56115</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="32" name="groomName">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E5F4B7A-1C2D-4666-A5C5-BB41EDA6AC25}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1774148" y="3358911"/>
-          <a:ext cx="1870200" cy="282068"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>	</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>67972</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>99445</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>159199</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>63210</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="33" name="brideName">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FDFDB630-FCBB-4352-888F-3126D10C062F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4917063" y="3372581"/>
-          <a:ext cx="1909636" cy="275493"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>33619</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>76323</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>75183</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>131506</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="34" name="letter">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E397648-E150-4A0B-9A39-B81E20A0ECB9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="33619" y="3972914"/>
-          <a:ext cx="7315200" cy="678637"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>	have successfully completed the mandatory Pre-Marriage Orientation and Counseling</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>	session held on [Insert Date] at the Municipal Hall, Solano, Nueva Vizcaya. This session 	covered:</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>104623</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>119257</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>519060</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>39963</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="35" name="TextBox 34">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5DCFE8B-D0F3-40F7-B102-62815B10B227}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2529168" y="4639302"/>
-          <a:ext cx="3445119" cy="855888"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr lvl="0" algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200"/>
-            <a:t>● </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Marriage and Relationships</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr lvl="0" algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200"/>
-            <a:t>● </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Responsible Parenthood</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr lvl="0" algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200"/>
-            <a:t>● </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Planning the Family</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr lvl="0" algn="l"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200"/>
-            <a:t>●</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Maternal, Neonatal, Child Health &amp; Nutrition</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="l"/>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>390867</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>120866</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>157370</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>113938</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="36" name="TextBox 35">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D282939A-4600-4BFB-B292-D860D0A80432}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1003780" y="6084344"/>
-          <a:ext cx="992329" cy="324377"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Control No: </a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>216324</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>117684</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>560295</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>104188</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="37" name="TextBox 36">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EE25D559-7F73-4658-BBD1-6020C170F3C8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4452148" y="5765449"/>
-          <a:ext cx="949088" cy="300268"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Issued On:</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>390697</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>99927</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>418948</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>87049</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="38" name="TextBox 37">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E62CF64B-9FB9-4184-9DE2-553E339E2F0C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="996833" y="6178609"/>
-          <a:ext cx="1846660" cy="298849"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>Signed:</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>8283</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>159023</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>72258</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>124387</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="39" name="TextBox 38">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C37CB8E-F3CE-4F7D-BA86-C99B747E6004}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8283" y="7447719"/>
-          <a:ext cx="7418932" cy="1621885"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>________________________		________________________</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> PMOC Team Representative		PMOC Team Representative</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>________________________		________________________</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> PMOC Team Representative		</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>PMOC Team Representative</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:endParaRPr lang="en-US" sz="1200">
-            <a:solidFill>
-              <a:schemeClr val="dk1"/>
-            </a:solidFill>
-            <a:effectLst/>
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>39414</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>110383</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>80977</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>102450</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="40" name="TextBox 39">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E5955BEB-BE4D-47C0-A0A4-13DB2843941E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="39414" y="10049513"/>
-          <a:ext cx="7396520" cy="489024"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
-            <a:lnSpc>
-              <a:spcPct val="100000"/>
-            </a:lnSpc>
-            <a:spcBef>
-              <a:spcPts val="0"/>
-            </a:spcBef>
-            <a:spcAft>
-              <a:spcPts val="0"/>
-            </a:spcAft>
-            <a:buClrTx/>
-            <a:buSzTx/>
-            <a:buFontTx/>
-            <a:buNone/>
-            <a:tabLst/>
-            <a:defRPr/>
-          </a:pPr>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Document Code: MCR.L.	   				 </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>    </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Control Number:</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Website: www.solano.gov.ph      		          Email: solanomcro@yahoo.com 	    </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Contact Number: 09175680286</a:t>
-          </a:r>
-          <a:br>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-          </a:br>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Facebook Pages: http://www.facebook/LguSolanoOfficialPage 	</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>                                   </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>http://www.facebook/OfficialLguSolanoFanPage</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="800">
-            <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>601201</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>122525</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>116896</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>114242</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="42" name="TextBox 41">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{534BB783-BC4C-C4D0-4B87-41A3A98FDF94}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1822133" y="5889480"/>
-          <a:ext cx="736627" cy="312103"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1200" b="1" u="none">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>PMOC-</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-US" sz="1200" u="none">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>511775</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>123304</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>541192</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>93541</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="43" name="yearToday">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B758C3B-694A-6C00-17D3-C826A8D9BA44}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2343173" y="5890259"/>
-          <a:ext cx="639883" cy="290623"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1200" b="1">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>355888</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>123824</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>510885</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>99579</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="44" name="controlNumber">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CF734D2-4961-06B4-9C0D-515521A38CF9}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2797752" y="5890779"/>
-          <a:ext cx="765463" cy="296141"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1200" b="1">
-            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>454602</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>125556</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>12989</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>99579</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="45" name="date">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5651F1E9-97C6-30E7-712B-BEB230B5C3DC}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5338329" y="5892511"/>
-          <a:ext cx="1389785" cy="294409"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="1100"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>165915</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>103038</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>39414</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>111674</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="46" name="yerdeyt">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9A697C84-D61A-40E0-5807-9B1632974564}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6275053" y="9956486"/>
-          <a:ext cx="484413" cy="172860"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="800">
-              <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>ormula</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>446689</xdr:colOff>
-      <xdr:row>60</xdr:row>
-      <xdr:rowOff>105104</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>553641</xdr:colOff>
-      <xdr:row>61</xdr:row>
-      <xdr:rowOff>105104</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="47" name="cN">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE8413F9-56E7-2639-83DF-CDE2644A20A3}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6518877" y="9749167"/>
-          <a:ext cx="714170" cy="160734"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="9525" cmpd="sng">
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="en-US" sz="800">
-            <a:latin typeface="Bookman Old Style" panose="02050604050505020204" pitchFamily="18" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -8997,917 +6770,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E47483-1312-4CC2-8463-3BBAA107E1DF}">
-  <dimension ref="A1:L64"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="159"/>
-      <c r="B1" s="159"/>
-      <c r="C1" s="159"/>
-      <c r="D1" s="159"/>
-      <c r="E1" s="159"/>
-      <c r="F1" s="159"/>
-      <c r="G1" s="159"/>
-      <c r="H1" s="159"/>
-      <c r="I1" s="159"/>
-      <c r="J1" s="159"/>
-      <c r="K1" s="159"/>
-      <c r="L1" s="159"/>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A2" s="159"/>
-      <c r="B2" s="159"/>
-      <c r="C2" s="159"/>
-      <c r="D2" s="159"/>
-      <c r="E2" s="159"/>
-      <c r="F2" s="159"/>
-      <c r="G2" s="159"/>
-      <c r="H2" s="159"/>
-      <c r="I2" s="159"/>
-      <c r="J2" s="159"/>
-      <c r="K2" s="159"/>
-      <c r="L2" s="159"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="159"/>
-      <c r="B3" s="159"/>
-      <c r="C3" s="159"/>
-      <c r="D3" s="159"/>
-      <c r="E3" s="159"/>
-      <c r="F3" s="159"/>
-      <c r="G3" s="159"/>
-      <c r="H3" s="159"/>
-      <c r="I3" s="159"/>
-      <c r="J3" s="159"/>
-      <c r="K3" s="159"/>
-      <c r="L3" s="159"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="159"/>
-      <c r="B4" s="159"/>
-      <c r="C4" s="159"/>
-      <c r="D4" s="159"/>
-      <c r="E4" s="159"/>
-      <c r="F4" s="159"/>
-      <c r="G4" s="159"/>
-      <c r="H4" s="159"/>
-      <c r="I4" s="159"/>
-      <c r="J4" s="159"/>
-      <c r="K4" s="159"/>
-      <c r="L4" s="159"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="159"/>
-      <c r="B5" s="159"/>
-      <c r="C5" s="159"/>
-      <c r="D5" s="159"/>
-      <c r="E5" s="159"/>
-      <c r="F5" s="159"/>
-      <c r="G5" s="159"/>
-      <c r="H5" s="159"/>
-      <c r="I5" s="159"/>
-      <c r="J5" s="159"/>
-      <c r="K5" s="159"/>
-      <c r="L5" s="159"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="159"/>
-      <c r="B6" s="159"/>
-      <c r="C6" s="159"/>
-      <c r="D6" s="159"/>
-      <c r="E6" s="159"/>
-      <c r="F6" s="159"/>
-      <c r="G6" s="159"/>
-      <c r="H6" s="159"/>
-      <c r="I6" s="159"/>
-      <c r="J6" s="159"/>
-      <c r="K6" s="159"/>
-      <c r="L6" s="159"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="159"/>
-      <c r="B7" s="159"/>
-      <c r="C7" s="159"/>
-      <c r="D7" s="159"/>
-      <c r="E7" s="159"/>
-      <c r="F7" s="159"/>
-      <c r="G7" s="159"/>
-      <c r="H7" s="159"/>
-      <c r="I7" s="159"/>
-      <c r="J7" s="159"/>
-      <c r="K7" s="159"/>
-      <c r="L7" s="159"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="159"/>
-      <c r="B8" s="159"/>
-      <c r="C8" s="159"/>
-      <c r="D8" s="159"/>
-      <c r="E8" s="159"/>
-      <c r="F8" s="159"/>
-      <c r="G8" s="159"/>
-      <c r="H8" s="159"/>
-      <c r="I8" s="159"/>
-      <c r="J8" s="159"/>
-      <c r="K8" s="159"/>
-      <c r="L8" s="159"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="159"/>
-      <c r="B9" s="159"/>
-      <c r="C9" s="159"/>
-      <c r="D9" s="159"/>
-      <c r="E9" s="159"/>
-      <c r="F9" s="159"/>
-      <c r="G9" s="159"/>
-      <c r="H9" s="159"/>
-      <c r="I9" s="159"/>
-      <c r="J9" s="159"/>
-      <c r="K9" s="159"/>
-      <c r="L9" s="159"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="159"/>
-      <c r="B10" s="159"/>
-      <c r="C10" s="159"/>
-      <c r="D10" s="159"/>
-      <c r="E10" s="159"/>
-      <c r="F10" s="159"/>
-      <c r="G10" s="159"/>
-      <c r="H10" s="159"/>
-      <c r="I10" s="159"/>
-      <c r="J10" s="159"/>
-      <c r="K10" s="159"/>
-      <c r="L10" s="159"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="159"/>
-      <c r="B11" s="159"/>
-      <c r="C11" s="159"/>
-      <c r="D11" s="159"/>
-      <c r="E11" s="159"/>
-      <c r="F11" s="159"/>
-      <c r="G11" s="159"/>
-      <c r="H11" s="159"/>
-      <c r="I11" s="159"/>
-      <c r="J11" s="159"/>
-      <c r="K11" s="159"/>
-      <c r="L11" s="159"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="159"/>
-      <c r="B12" s="159"/>
-      <c r="C12" s="159"/>
-      <c r="D12" s="159"/>
-      <c r="E12" s="159"/>
-      <c r="F12" s="159"/>
-      <c r="G12" s="159"/>
-      <c r="H12" s="159"/>
-      <c r="I12" s="159"/>
-      <c r="J12" s="159"/>
-      <c r="K12" s="159"/>
-      <c r="L12" s="159"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="159"/>
-      <c r="B13" s="159"/>
-      <c r="C13" s="159"/>
-      <c r="D13" s="159"/>
-      <c r="E13" s="159"/>
-      <c r="F13" s="159"/>
-      <c r="G13" s="159"/>
-      <c r="H13" s="159"/>
-      <c r="I13" s="159"/>
-      <c r="J13" s="159"/>
-      <c r="K13" s="159"/>
-      <c r="L13" s="159"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="159"/>
-      <c r="B14" s="159"/>
-      <c r="C14" s="159"/>
-      <c r="D14" s="159"/>
-      <c r="E14" s="159"/>
-      <c r="F14" s="159"/>
-      <c r="G14" s="159"/>
-      <c r="H14" s="159"/>
-      <c r="I14" s="159"/>
-      <c r="J14" s="159"/>
-      <c r="K14" s="159"/>
-      <c r="L14" s="159"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="159"/>
-      <c r="B15" s="159"/>
-      <c r="C15" s="159"/>
-      <c r="D15" s="159"/>
-      <c r="E15" s="159"/>
-      <c r="F15" s="159"/>
-      <c r="G15" s="159"/>
-      <c r="H15" s="159"/>
-      <c r="I15" s="159"/>
-      <c r="J15" s="159"/>
-      <c r="K15" s="159"/>
-      <c r="L15" s="159"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="159"/>
-      <c r="B16" s="159"/>
-      <c r="C16" s="159"/>
-      <c r="D16" s="159"/>
-      <c r="E16" s="159"/>
-      <c r="F16" s="159"/>
-      <c r="G16" s="159"/>
-      <c r="H16" s="159"/>
-      <c r="I16" s="159"/>
-      <c r="J16" s="159"/>
-      <c r="K16" s="159"/>
-      <c r="L16" s="159"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="159"/>
-      <c r="B17" s="159"/>
-      <c r="C17" s="159"/>
-      <c r="D17" s="159"/>
-      <c r="E17" s="159"/>
-      <c r="F17" s="159"/>
-      <c r="G17" s="159"/>
-      <c r="H17" s="159"/>
-      <c r="I17" s="159"/>
-      <c r="J17" s="159"/>
-      <c r="K17" s="159"/>
-      <c r="L17" s="159"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="159"/>
-      <c r="B18" s="159"/>
-      <c r="C18" s="159"/>
-      <c r="D18" s="159"/>
-      <c r="E18" s="159"/>
-      <c r="F18" s="159"/>
-      <c r="G18" s="159"/>
-      <c r="H18" s="159"/>
-      <c r="I18" s="159"/>
-      <c r="J18" s="159"/>
-      <c r="K18" s="159"/>
-      <c r="L18" s="159"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="159"/>
-      <c r="B19" s="159"/>
-      <c r="C19" s="159"/>
-      <c r="D19" s="159"/>
-      <c r="E19" s="159"/>
-      <c r="F19" s="159"/>
-      <c r="G19" s="159"/>
-      <c r="H19" s="159"/>
-      <c r="I19" s="159"/>
-      <c r="J19" s="159"/>
-      <c r="K19" s="159"/>
-      <c r="L19" s="159"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="159"/>
-      <c r="B20" s="159"/>
-      <c r="C20" s="159"/>
-      <c r="D20" s="159"/>
-      <c r="E20" s="159"/>
-      <c r="F20" s="159"/>
-      <c r="G20" s="159"/>
-      <c r="H20" s="159"/>
-      <c r="I20" s="159"/>
-      <c r="J20" s="159"/>
-      <c r="K20" s="159"/>
-      <c r="L20" s="159"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A21" s="159"/>
-      <c r="B21" s="159"/>
-      <c r="C21" s="159"/>
-      <c r="D21" s="159"/>
-      <c r="E21" s="159"/>
-      <c r="F21" s="159"/>
-      <c r="G21" s="159"/>
-      <c r="H21" s="159"/>
-      <c r="I21" s="159"/>
-      <c r="J21" s="159"/>
-      <c r="K21" s="159"/>
-      <c r="L21" s="159"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="159"/>
-      <c r="B22" s="159"/>
-      <c r="C22" s="159"/>
-      <c r="D22" s="159"/>
-      <c r="E22" s="159"/>
-      <c r="F22" s="159"/>
-      <c r="G22" s="159"/>
-      <c r="H22" s="159"/>
-      <c r="I22" s="159"/>
-      <c r="J22" s="159"/>
-      <c r="K22" s="159"/>
-      <c r="L22" s="159"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="159"/>
-      <c r="B23" s="159"/>
-      <c r="C23" s="159"/>
-      <c r="D23" s="159"/>
-      <c r="E23" s="159"/>
-      <c r="F23" s="159"/>
-      <c r="G23" s="159"/>
-      <c r="H23" s="159"/>
-      <c r="I23" s="159"/>
-      <c r="J23" s="159"/>
-      <c r="K23" s="159"/>
-      <c r="L23" s="159"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="159"/>
-      <c r="B24" s="159"/>
-      <c r="C24" s="159"/>
-      <c r="D24" s="159"/>
-      <c r="E24" s="159"/>
-      <c r="F24" s="159"/>
-      <c r="G24" s="159"/>
-      <c r="H24" s="159"/>
-      <c r="I24" s="159"/>
-      <c r="J24" s="159"/>
-      <c r="K24" s="159"/>
-      <c r="L24" s="159"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="159"/>
-      <c r="B25" s="159"/>
-      <c r="C25" s="159"/>
-      <c r="D25" s="159"/>
-      <c r="E25" s="159"/>
-      <c r="F25" s="159"/>
-      <c r="G25" s="159"/>
-      <c r="H25" s="159"/>
-      <c r="I25" s="159"/>
-      <c r="J25" s="159"/>
-      <c r="K25" s="159"/>
-      <c r="L25" s="159"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A26" s="159"/>
-      <c r="B26" s="159"/>
-      <c r="C26" s="159"/>
-      <c r="D26" s="159"/>
-      <c r="E26" s="159"/>
-      <c r="F26" s="159"/>
-      <c r="G26" s="159"/>
-      <c r="H26" s="159"/>
-      <c r="I26" s="159"/>
-      <c r="J26" s="159"/>
-      <c r="K26" s="159"/>
-      <c r="L26" s="159"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="159"/>
-      <c r="B27" s="159"/>
-      <c r="C27" s="159"/>
-      <c r="D27" s="159"/>
-      <c r="E27" s="159"/>
-      <c r="F27" s="159"/>
-      <c r="G27" s="159"/>
-      <c r="H27" s="159"/>
-      <c r="I27" s="159"/>
-      <c r="J27" s="159"/>
-      <c r="K27" s="159"/>
-      <c r="L27" s="159"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="159"/>
-      <c r="B28" s="159"/>
-      <c r="C28" s="159"/>
-      <c r="D28" s="159"/>
-      <c r="E28" s="159"/>
-      <c r="F28" s="159"/>
-      <c r="G28" s="159"/>
-      <c r="H28" s="159"/>
-      <c r="I28" s="159"/>
-      <c r="J28" s="159"/>
-      <c r="K28" s="159"/>
-      <c r="L28" s="159"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="159"/>
-      <c r="B29" s="159"/>
-      <c r="C29" s="159"/>
-      <c r="D29" s="159"/>
-      <c r="E29" s="159"/>
-      <c r="F29" s="159"/>
-      <c r="G29" s="159"/>
-      <c r="H29" s="159"/>
-      <c r="I29" s="159"/>
-      <c r="J29" s="159"/>
-      <c r="K29" s="159"/>
-      <c r="L29" s="159"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="159"/>
-      <c r="B30" s="159"/>
-      <c r="C30" s="159"/>
-      <c r="D30" s="159"/>
-      <c r="E30" s="159"/>
-      <c r="F30" s="159"/>
-      <c r="G30" s="159"/>
-      <c r="H30" s="159"/>
-      <c r="I30" s="159"/>
-      <c r="J30" s="159"/>
-      <c r="K30" s="159"/>
-      <c r="L30" s="159"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="159"/>
-      <c r="B31" s="159"/>
-      <c r="C31" s="159"/>
-      <c r="D31" s="159"/>
-      <c r="E31" s="159"/>
-      <c r="F31" s="159"/>
-      <c r="G31" s="159"/>
-      <c r="H31" s="159"/>
-      <c r="I31" s="159"/>
-      <c r="J31" s="159"/>
-      <c r="K31" s="159"/>
-      <c r="L31" s="159"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A32" s="159"/>
-      <c r="B32" s="159"/>
-      <c r="C32" s="159"/>
-      <c r="D32" s="159"/>
-      <c r="E32" s="159"/>
-      <c r="F32" s="159"/>
-      <c r="G32" s="159"/>
-      <c r="H32" s="159"/>
-      <c r="I32" s="159"/>
-      <c r="J32" s="159"/>
-      <c r="K32" s="159"/>
-      <c r="L32" s="159"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A33" s="159"/>
-      <c r="B33" s="159"/>
-      <c r="C33" s="159"/>
-      <c r="D33" s="159"/>
-      <c r="E33" s="159"/>
-      <c r="F33" s="159"/>
-      <c r="G33" s="159"/>
-      <c r="H33" s="159"/>
-      <c r="I33" s="159"/>
-      <c r="J33" s="159"/>
-      <c r="K33" s="159"/>
-      <c r="L33" s="159"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" s="159"/>
-      <c r="B34" s="159"/>
-      <c r="C34" s="159"/>
-      <c r="D34" s="159"/>
-      <c r="E34" s="159"/>
-      <c r="F34" s="159"/>
-      <c r="G34" s="159"/>
-      <c r="H34" s="159"/>
-      <c r="I34" s="159"/>
-      <c r="J34" s="159"/>
-      <c r="K34" s="159"/>
-      <c r="L34" s="159"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="159"/>
-      <c r="B35" s="159"/>
-      <c r="C35" s="159"/>
-      <c r="D35" s="159"/>
-      <c r="E35" s="159"/>
-      <c r="F35" s="159"/>
-      <c r="G35" s="159"/>
-      <c r="H35" s="159"/>
-      <c r="I35" s="159"/>
-      <c r="J35" s="159"/>
-      <c r="K35" s="159"/>
-      <c r="L35" s="159"/>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A36" s="159"/>
-      <c r="B36" s="159"/>
-      <c r="C36" s="159"/>
-      <c r="D36" s="159"/>
-      <c r="E36" s="159"/>
-      <c r="F36" s="159"/>
-      <c r="G36" s="159"/>
-      <c r="H36" s="159"/>
-      <c r="I36" s="159"/>
-      <c r="J36" s="159"/>
-      <c r="K36" s="159"/>
-      <c r="L36" s="159"/>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A37" s="159"/>
-      <c r="B37" s="159"/>
-      <c r="C37" s="159"/>
-      <c r="D37" s="159"/>
-      <c r="E37" s="159"/>
-      <c r="F37" s="159"/>
-      <c r="G37" s="159"/>
-      <c r="H37" s="159"/>
-      <c r="I37" s="159"/>
-      <c r="J37" s="159"/>
-      <c r="K37" s="159"/>
-      <c r="L37" s="159"/>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A38" s="159"/>
-      <c r="B38" s="159"/>
-      <c r="C38" s="159"/>
-      <c r="D38" s="159"/>
-      <c r="E38" s="159"/>
-      <c r="F38" s="159"/>
-      <c r="G38" s="159"/>
-      <c r="H38" s="159"/>
-      <c r="I38" s="159"/>
-      <c r="J38" s="159"/>
-      <c r="K38" s="159"/>
-      <c r="L38" s="159"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A39" s="159"/>
-      <c r="B39" s="159"/>
-      <c r="C39" s="159"/>
-      <c r="D39" s="159"/>
-      <c r="E39" s="159"/>
-      <c r="F39" s="159"/>
-      <c r="G39" s="159"/>
-      <c r="H39" s="159"/>
-      <c r="I39" s="159"/>
-      <c r="J39" s="159"/>
-      <c r="K39" s="159"/>
-      <c r="L39" s="159"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A40" s="159"/>
-      <c r="B40" s="159"/>
-      <c r="C40" s="159"/>
-      <c r="D40" s="159"/>
-      <c r="E40" s="159"/>
-      <c r="F40" s="159"/>
-      <c r="G40" s="159"/>
-      <c r="H40" s="159"/>
-      <c r="I40" s="159"/>
-      <c r="J40" s="159"/>
-      <c r="K40" s="159"/>
-      <c r="L40" s="159"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A41" s="159"/>
-      <c r="B41" s="159"/>
-      <c r="C41" s="159"/>
-      <c r="D41" s="159"/>
-      <c r="E41" s="159"/>
-      <c r="F41" s="159"/>
-      <c r="G41" s="159"/>
-      <c r="H41" s="159"/>
-      <c r="I41" s="159"/>
-      <c r="J41" s="159"/>
-      <c r="K41" s="159"/>
-      <c r="L41" s="159"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A42" s="159"/>
-      <c r="B42" s="159"/>
-      <c r="C42" s="159"/>
-      <c r="D42" s="159"/>
-      <c r="E42" s="159"/>
-      <c r="F42" s="159"/>
-      <c r="G42" s="159"/>
-      <c r="H42" s="159"/>
-      <c r="I42" s="159"/>
-      <c r="J42" s="159"/>
-      <c r="K42" s="159"/>
-      <c r="L42" s="159"/>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A43" s="159"/>
-      <c r="B43" s="159"/>
-      <c r="C43" s="159"/>
-      <c r="D43" s="159"/>
-      <c r="E43" s="159"/>
-      <c r="F43" s="159"/>
-      <c r="G43" s="159"/>
-      <c r="H43" s="159"/>
-      <c r="I43" s="159"/>
-      <c r="J43" s="159"/>
-      <c r="K43" s="159"/>
-      <c r="L43" s="159"/>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A44" s="159"/>
-      <c r="B44" s="159"/>
-      <c r="C44" s="159"/>
-      <c r="D44" s="159"/>
-      <c r="E44" s="159"/>
-      <c r="F44" s="159"/>
-      <c r="G44" s="159"/>
-      <c r="H44" s="159"/>
-      <c r="I44" s="159"/>
-      <c r="J44" s="159"/>
-      <c r="K44" s="159"/>
-      <c r="L44" s="159"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A45" s="159"/>
-      <c r="B45" s="159"/>
-      <c r="C45" s="159"/>
-      <c r="D45" s="159"/>
-      <c r="E45" s="159"/>
-      <c r="F45" s="159"/>
-      <c r="G45" s="159"/>
-      <c r="H45" s="159"/>
-      <c r="I45" s="159"/>
-      <c r="J45" s="159"/>
-      <c r="K45" s="159"/>
-      <c r="L45" s="159"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A46" s="159"/>
-      <c r="B46" s="159"/>
-      <c r="C46" s="159"/>
-      <c r="D46" s="159"/>
-      <c r="E46" s="159"/>
-      <c r="F46" s="159"/>
-      <c r="G46" s="159"/>
-      <c r="H46" s="159"/>
-      <c r="I46" s="159"/>
-      <c r="J46" s="159"/>
-      <c r="K46" s="159"/>
-      <c r="L46" s="159"/>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A47" s="159"/>
-      <c r="B47" s="159"/>
-      <c r="C47" s="159"/>
-      <c r="D47" s="159"/>
-      <c r="E47" s="159"/>
-      <c r="F47" s="159"/>
-      <c r="G47" s="159"/>
-      <c r="H47" s="159"/>
-      <c r="I47" s="159"/>
-      <c r="J47" s="159"/>
-      <c r="K47" s="159"/>
-      <c r="L47" s="159"/>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A48" s="159"/>
-      <c r="B48" s="159"/>
-      <c r="C48" s="159"/>
-      <c r="D48" s="159"/>
-      <c r="E48" s="159"/>
-      <c r="F48" s="159"/>
-      <c r="G48" s="159"/>
-      <c r="H48" s="159"/>
-      <c r="I48" s="159"/>
-      <c r="J48" s="159"/>
-      <c r="K48" s="159"/>
-      <c r="L48" s="159"/>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A49" s="159"/>
-      <c r="B49" s="159"/>
-      <c r="C49" s="159"/>
-      <c r="D49" s="159"/>
-      <c r="E49" s="159"/>
-      <c r="F49" s="159"/>
-      <c r="G49" s="159"/>
-      <c r="H49" s="159"/>
-      <c r="I49" s="159"/>
-      <c r="J49" s="159"/>
-      <c r="K49" s="159"/>
-      <c r="L49" s="159"/>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A50" s="159"/>
-      <c r="B50" s="159"/>
-      <c r="C50" s="159"/>
-      <c r="D50" s="159"/>
-      <c r="E50" s="159"/>
-      <c r="F50" s="159"/>
-      <c r="G50" s="159"/>
-      <c r="H50" s="159"/>
-      <c r="I50" s="159"/>
-      <c r="J50" s="159"/>
-      <c r="K50" s="159"/>
-      <c r="L50" s="159"/>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A51" s="159"/>
-      <c r="B51" s="159"/>
-      <c r="C51" s="159"/>
-      <c r="D51" s="159"/>
-      <c r="E51" s="159"/>
-      <c r="F51" s="159"/>
-      <c r="G51" s="159"/>
-      <c r="H51" s="159"/>
-      <c r="I51" s="159"/>
-      <c r="J51" s="159"/>
-      <c r="K51" s="159"/>
-      <c r="L51" s="159"/>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A52" s="159"/>
-      <c r="B52" s="159"/>
-      <c r="C52" s="159"/>
-      <c r="D52" s="159"/>
-      <c r="E52" s="159"/>
-      <c r="F52" s="159"/>
-      <c r="G52" s="159"/>
-      <c r="H52" s="159"/>
-      <c r="I52" s="159"/>
-      <c r="J52" s="159"/>
-      <c r="K52" s="159"/>
-      <c r="L52" s="159"/>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A53" s="159"/>
-      <c r="B53" s="159"/>
-      <c r="C53" s="159"/>
-      <c r="D53" s="159"/>
-      <c r="E53" s="159"/>
-      <c r="F53" s="159"/>
-      <c r="G53" s="159"/>
-      <c r="H53" s="159"/>
-      <c r="I53" s="159"/>
-      <c r="J53" s="159"/>
-      <c r="K53" s="159"/>
-      <c r="L53" s="159"/>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A54" s="159"/>
-      <c r="B54" s="159"/>
-      <c r="C54" s="159"/>
-      <c r="D54" s="159"/>
-      <c r="E54" s="159"/>
-      <c r="F54" s="159"/>
-      <c r="G54" s="159"/>
-      <c r="H54" s="159"/>
-      <c r="I54" s="159"/>
-      <c r="J54" s="159"/>
-      <c r="K54" s="159"/>
-      <c r="L54" s="159"/>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A55" s="159"/>
-      <c r="B55" s="159"/>
-      <c r="C55" s="159"/>
-      <c r="D55" s="159"/>
-      <c r="E55" s="159"/>
-      <c r="F55" s="159"/>
-      <c r="G55" s="159"/>
-      <c r="H55" s="159"/>
-      <c r="I55" s="159"/>
-      <c r="J55" s="159"/>
-      <c r="K55" s="159"/>
-      <c r="L55" s="159"/>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A56" s="159"/>
-      <c r="B56" s="159"/>
-      <c r="C56" s="159"/>
-      <c r="D56" s="159"/>
-      <c r="E56" s="159"/>
-      <c r="F56" s="159"/>
-      <c r="G56" s="159"/>
-      <c r="H56" s="159"/>
-      <c r="I56" s="159"/>
-      <c r="J56" s="159"/>
-      <c r="K56" s="159"/>
-      <c r="L56" s="159"/>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A57" s="159"/>
-      <c r="B57" s="159"/>
-      <c r="C57" s="159"/>
-      <c r="D57" s="159"/>
-      <c r="E57" s="159"/>
-      <c r="F57" s="159"/>
-      <c r="G57" s="159"/>
-      <c r="H57" s="159"/>
-      <c r="I57" s="159"/>
-      <c r="J57" s="159"/>
-      <c r="K57" s="159"/>
-      <c r="L57" s="159"/>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A58" s="159"/>
-      <c r="B58" s="159"/>
-      <c r="C58" s="159"/>
-      <c r="D58" s="159"/>
-      <c r="E58" s="159"/>
-      <c r="F58" s="159"/>
-      <c r="G58" s="159"/>
-      <c r="H58" s="159"/>
-      <c r="I58" s="159"/>
-      <c r="J58" s="159"/>
-      <c r="K58" s="159"/>
-      <c r="L58" s="159"/>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A59" s="159"/>
-      <c r="B59" s="159"/>
-      <c r="C59" s="159"/>
-      <c r="D59" s="159"/>
-      <c r="E59" s="159"/>
-      <c r="F59" s="159"/>
-      <c r="G59" s="159"/>
-      <c r="H59" s="159"/>
-      <c r="I59" s="159"/>
-      <c r="J59" s="159"/>
-      <c r="K59" s="159"/>
-      <c r="L59" s="159"/>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A60" s="159"/>
-      <c r="B60" s="159"/>
-      <c r="C60" s="159"/>
-      <c r="D60" s="159"/>
-      <c r="E60" s="159"/>
-      <c r="F60" s="159"/>
-      <c r="G60" s="159"/>
-      <c r="H60" s="159"/>
-      <c r="I60" s="159"/>
-      <c r="J60" s="159"/>
-      <c r="K60" s="159"/>
-      <c r="L60" s="159"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A61" s="159"/>
-      <c r="B61" s="159"/>
-      <c r="C61" s="159"/>
-      <c r="D61" s="159"/>
-      <c r="E61" s="159"/>
-      <c r="F61" s="159"/>
-      <c r="G61" s="159"/>
-      <c r="H61" s="159"/>
-      <c r="I61" s="159"/>
-      <c r="J61" s="159"/>
-      <c r="K61" s="159"/>
-      <c r="L61" s="159"/>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A62" s="159"/>
-      <c r="B62" s="159"/>
-      <c r="C62" s="159"/>
-      <c r="D62" s="159"/>
-      <c r="E62" s="159"/>
-      <c r="F62" s="159"/>
-      <c r="G62" s="159"/>
-      <c r="H62" s="159"/>
-      <c r="I62" s="159"/>
-      <c r="J62" s="159"/>
-      <c r="K62" s="159"/>
-      <c r="L62" s="159"/>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A63" s="159"/>
-      <c r="B63" s="159"/>
-      <c r="C63" s="159"/>
-      <c r="D63" s="159"/>
-      <c r="E63" s="159"/>
-      <c r="F63" s="159"/>
-      <c r="G63" s="159"/>
-      <c r="H63" s="159"/>
-      <c r="I63" s="159"/>
-      <c r="J63" s="159"/>
-      <c r="K63" s="159"/>
-      <c r="L63" s="159"/>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A64" s="159"/>
-      <c r="B64" s="159"/>
-      <c r="C64" s="159"/>
-      <c r="D64" s="159"/>
-      <c r="E64" s="159"/>
-      <c r="F64" s="159"/>
-      <c r="G64" s="159"/>
-      <c r="H64" s="159"/>
-      <c r="I64" s="159"/>
-      <c r="J64" s="159"/>
-      <c r="K64" s="159"/>
-      <c r="L64" s="159"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:L64"/>
-  </mergeCells>
-  <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet3"/>

</xml_diff>